<commit_message>
Update VNSH03 hàn thêm M2 NVMe.xlsx
</commit_message>
<xml_diff>
--- a/5. Other/VNSH03 hàn thêm M2 NVMe.xlsx
+++ b/5. Other/VNSH03 hàn thêm M2 NVMe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VNET\5. Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA4CAC68-DBF3-4DA1-82D4-19081CC88DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4109B855-4368-464F-9CCE-7C09343819B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{EC3BDDC8-0DA6-465B-868D-CE194108D9E1}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="47">
   <si>
     <t>200 Thiết bị VNSH03 hàn thêm khe M2</t>
   </si>
@@ -1159,11 +1159,17 @@
       <c r="B31" s="7">
         <v>46315</v>
       </c>
+      <c r="C31" s="7">
+        <v>46315</v>
+      </c>
       <c r="D31" s="2" t="s">
         <v>46</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>39</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>